<commit_message>
fix: standardise Gold intermediate SQL aliases to snake case
</commit_message>
<xml_diff>
--- a/project X/configuration/Dashboard Legend.xlsx
+++ b/project X/configuration/Dashboard Legend.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R6cdac514a4af4c57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="R2e3621ab31c44813"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="Rc4439a7b09004254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R29673c5aae9e420f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="Rfc5658c09e2e4a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="Rfa46288eb3004e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="R4a1ec47b108f4369"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -874,7 +875,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -914,8 +915,26 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF92400E"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF9A3412"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF374151"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1017,8 +1036,48 @@
         <x:fgColor rgb="FF4B5563"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF200"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDE7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F2937"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4B5563"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFEDD5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F4F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="13">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -1110,13 +1169,31 @@
         <x:color rgb="FFD1D5DB"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="114">
+  <x:cellXfs count="148">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1347,13 +1424,81 @@
     <x:xf numFmtId="0" fontId="6" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="26" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="3">
     <x:cellStyle name="Bad" xfId="2"/>
     <x:cellStyle name="Good" xfId="1"/>
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="36">
+  <x:dxfs count="48">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1657,7 +1802,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1668,7 +1813,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -1679,7 +1824,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -1690,7 +1835,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1701,7 +1846,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -1712,7 +1857,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -1723,7 +1868,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1734,7 +1879,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -1745,8 +1890,139 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9A3412"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFEDD5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1D4ED8"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9A3412"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFEDD5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1D4ED8"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1F4D2E"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1769,7 +2045,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ActiveGoldKpis" displayName="ActiveGoldKpis" ref="A4:H112" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ActiveGoldKpis" displayName="ActiveGoldKpis" ref="A4:H113" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Gold KPI ID"/>
     <x:tableColumn id="2" name="Business area"/>
@@ -1794,6 +2070,22 @@
     <x:tableColumn id="5" name="Requirement IDs"/>
     <x:tableColumn id="6" name="Status"/>
     <x:tableColumn id="7" name="Reason / next Gold-model change"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="GoldSourceCoverage" displayName="GoldSourceCoverage" ref="A4:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Requirement / capability"/>
+    <x:tableColumn id="2" name="Required source entity / extract"/>
+    <x:tableColumn id="3" name="Expected Bronze → Silver table"/>
+    <x:tableColumn id="4" name="Fields needed"/>
+    <x:tableColumn id="5" name="Source / Silver evidence"/>
+    <x:tableColumn id="6" name="Current Gold publication"/>
+    <x:tableColumn id="7" name="Gold coverage"/>
+    <x:tableColumn id="8" name="Action / conclusion"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -5362,7 +5654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b7ab53a1c44496f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6548377d9a764079"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8264,14 +8556,30 @@
       </x:c>
     </x:row>
     <x:row r="113" ht="14.5" hidden="0" customHeight="1">
-      <x:c r="A113"/>
-      <x:c r="B113"/>
-      <x:c r="C113"/>
-      <x:c r="D113"/>
-      <x:c r="E113"/>
-      <x:c r="F113"/>
-      <x:c r="G113"/>
-      <x:c r="H113"/>
+      <x:c r="A113" t="str">
+        <x:v>GOLD-KPI-109</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>Message activity proxy</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>Provider Messages Sent</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>KPI-110 proxy</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>R14</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>fact_referral_lifecycle_event</x:v>
+      </x:c>
+      <x:c r="G113" s="134" t="str">
+        <x:v>Proxy only</x:v>
+      </x:c>
+      <x:c r="H113" t="str">
+        <x:v>IPA, cost and referral-lifecycle measures</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="14.5" hidden="0" customHeight="1">
       <x:c r="A114"/>
@@ -8495,19 +8803,19 @@
         <x:v>Provider messages</x:v>
       </x:c>
       <x:c r="C124" s="42" t="str">
-        <x:v>Message volume, response time and unread priorities (KPI-110–112)</x:v>
+        <x:v>Message response-time and unread-priority KPIs (KPI-111–112)</x:v>
       </x:c>
       <x:c r="D124" s="42" t="str">
-        <x:v>KPI-110–112</x:v>
+        <x:v>KPI-111–112</x:v>
       </x:c>
       <x:c r="E124" s="42" t="str">
         <x:v>R14</x:v>
       </x:c>
-      <x:c r="F124" s="42" t="str">
-        <x:v>Needs Gold data</x:v>
+      <x:c r="F124" s="136" t="str">
+        <x:v>Silver available — not promoted</x:v>
       </x:c>
       <x:c r="G124" s="43" t="str">
-        <x:v>No provider-message or message-status fact is published in active Gold.</x:v>
+        <x:v>Provider Messages Sent is a lifecycle-event proxy. Build detailed message and message-status Gold facts for response-time and unread analysis.</x:v>
       </x:c>
       <x:c r="H124"/>
     </x:row>
@@ -9131,8 +9439,643 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re173117eeb7d4736"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ed19f79dd354ece"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e89323d8ede4065"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2575e3d04b3646af"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="45" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="64" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="116" t="str">
+        <x:v>Requirement source-file coverage and Gold promotion status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
+      <x:c r="A2" s="139" t="str">
+        <x:v>Published Power BI DAX may use only rows marked Yes. All other rows are source lineage or a Gold-promotion roadmap, not permitted KPI sources.</x:v>
+      </x:c>
+      <x:c r="B2" s="139"/>
+      <x:c r="C2" s="139"/>
+      <x:c r="D2" s="139"/>
+      <x:c r="E2" s="139"/>
+      <x:c r="F2" s="139"/>
+      <x:c r="G2" s="139"/>
+      <x:c r="H2" s="139"/>
+      <x:c r="I2" s="139"/>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="126" t="str">
+        <x:v>Requirement / capability</x:v>
+      </x:c>
+      <x:c r="B4" s="126" t="str">
+        <x:v>Required source entity / extract</x:v>
+      </x:c>
+      <x:c r="C4" s="126" t="str">
+        <x:v>Expected Bronze → Silver table</x:v>
+      </x:c>
+      <x:c r="D4" s="126" t="str">
+        <x:v>Fields needed</x:v>
+      </x:c>
+      <x:c r="E4" s="126" t="str">
+        <x:v>Source / Silver evidence</x:v>
+      </x:c>
+      <x:c r="F4" s="126" t="str">
+        <x:v>Current Gold publication</x:v>
+      </x:c>
+      <x:c r="G4" s="126" t="str">
+        <x:v>Gold coverage</x:v>
+      </x:c>
+      <x:c r="H4" s="126" t="str">
+        <x:v>Action / conclusion</x:v>
+      </x:c>
+      <x:c r="I4" s="146" t="str">
+        <x:v>KPI DAX eligibility</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="38" t="str">
+        <x:v>Referral core</x:v>
+      </x:c>
+      <x:c r="B5" s="39" t="str">
+        <x:v>referral</x:v>
+      </x:c>
+      <x:c r="C5" s="39" t="str">
+        <x:v>bronze.referral → silver.referral</x:v>
+      </x:c>
+      <x:c r="D5" s="39" t="str">
+        <x:v>referral_id, referral_created_date, required_start_date, referral_status, referral_modified_date</x:v>
+      </x:c>
+      <x:c r="E5" s="39" t="str">
+        <x:v>Contracted and used</x:v>
+      </x:c>
+      <x:c r="F5" s="39" t="str">
+        <x:v>gold.fact_referral; gold.fact_referral_snapshot; dim_referral_status; dim_placement_type</x:v>
+      </x:c>
+      <x:c r="G5" s="39" t="str">
+        <x:v>Published in Gold</x:v>
+      </x:c>
+      <x:c r="H5" s="40" t="str">
+        <x:v>Core referral KPIs and snapshots are supported.</x:v>
+      </x:c>
+      <x:c r="I5" s="147" t="str">
+        <x:v>Yes — Gold field</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="41" t="str">
+        <x:v>Referral-provider engagement</x:v>
+      </x:c>
+      <x:c r="B6" s="42" t="str">
+        <x:v>referral_provider</x:v>
+      </x:c>
+      <x:c r="C6" s="42" t="str">
+        <x:v>bronze.referral_provider → silver.referral_provider</x:v>
+      </x:c>
+      <x:c r="D6" s="42" t="str">
+        <x:v>referral_provider_id, referral_id, provider_id, is_excluded, is_declined, is_cancelled, is_closed</x:v>
+      </x:c>
+      <x:c r="E6" s="42" t="str">
+        <x:v>Contracted and used</x:v>
+      </x:c>
+      <x:c r="F6" s="42" t="str">
+        <x:v>gold.fact_referral_provider</x:v>
+      </x:c>
+      <x:c r="G6" s="42" t="str">
+        <x:v>Published in Gold</x:v>
+      </x:c>
+      <x:c r="H6" s="43" t="str">
+        <x:v>Provider assignment and decline-rate measures are supported.</x:v>
+      </x:c>
+      <x:c r="I6" s="147" t="str">
+        <x:v>Yes — Gold field</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="41" t="str">
+        <x:v>Provider offers</x:v>
+      </x:c>
+      <x:c r="B7" s="42" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="C7" s="42" t="str">
+        <x:v>bronze.offer → silver.offer</x:v>
+      </x:c>
+      <x:c r="D7" s="42" t="str">
+        <x:v>offer_id, referral_provider_id, offer_status, offer_date, last_modified_date, fees, decline reasons</x:v>
+      </x:c>
+      <x:c r="E7" s="42" t="str">
+        <x:v>Contracted and used</x:v>
+      </x:c>
+      <x:c r="F7" s="42" t="str">
+        <x:v>gold.fact_offer</x:v>
+      </x:c>
+      <x:c r="G7" s="42" t="str">
+        <x:v>Published in Gold</x:v>
+      </x:c>
+      <x:c r="H7" s="43" t="str">
+        <x:v>Offer, decision, age, cost and rejection-reason measures are supported.</x:v>
+      </x:c>
+      <x:c r="I7" s="147" t="str">
+        <x:v>Yes — Gold field</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A8" s="41" t="str">
+        <x:v>IPA core</x:v>
+      </x:c>
+      <x:c r="B8" s="42" t="str">
+        <x:v>ipa</x:v>
+      </x:c>
+      <x:c r="C8" s="42" t="str">
+        <x:v>bronze.ipa → silver.ipa</x:v>
+      </x:c>
+      <x:c r="D8" s="42" t="str">
+        <x:v>ipa_id, referral_id, offer_id, created_datetime, placement_admission_date, costs_total_weekly_fee, status, closed</x:v>
+      </x:c>
+      <x:c r="E8" s="42" t="str">
+        <x:v>Contracted and used</x:v>
+      </x:c>
+      <x:c r="F8" s="42" t="str">
+        <x:v>gold.fct_ipa</x:v>
+      </x:c>
+      <x:c r="G8" s="42" t="str">
+        <x:v>Published in Gold</x:v>
+      </x:c>
+      <x:c r="H8" s="43" t="str">
+        <x:v>IPA volume, placement status and active weekly-cost measures are supported.</x:v>
+      </x:c>
+      <x:c r="I8" s="147" t="str">
+        <x:v>Yes — Gold field</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="41" t="str">
+        <x:v>IPA signatures</x:v>
+      </x:c>
+      <x:c r="B9" s="42" t="str">
+        <x:v>ipa</x:v>
+      </x:c>
+      <x:c r="C9" s="42" t="str">
+        <x:v>bronze.ipa → silver.ipa</x:v>
+      </x:c>
+      <x:c r="D9" s="42" t="str">
+        <x:v>signed_by_local_authority, signed_datetime_for_local_authority, signed_by_provider, signed_datetime_for_provider</x:v>
+      </x:c>
+      <x:c r="E9" s="42" t="str">
+        <x:v>Contracted; not selected by the Gold IPA query</x:v>
+      </x:c>
+      <x:c r="F9" s="42" t="str">
+        <x:v>fact_referral has ipa_2_signatures proxy only</x:v>
+      </x:c>
+      <x:c r="G9" s="42" t="str">
+        <x:v>Silver available — not promoted</x:v>
+      </x:c>
+      <x:c r="H9" s="43" t="str">
+        <x:v>No new source file is needed. Extend gold.fct_ipa with signature fields for true IPA-grain completion KPIs.</x:v>
+      </x:c>
+      <x:c r="I9" s="147" t="str">
+        <x:v>No — promote IPA fields</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A10" s="41" t="str">
+        <x:v>IPA payment and invoice</x:v>
+      </x:c>
+      <x:c r="B10" s="42" t="str">
+        <x:v>ipa</x:v>
+      </x:c>
+      <x:c r="C10" s="42" t="str">
+        <x:v>bronze.ipa → silver.ipa</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="str">
+        <x:v>payment_method, invoice fields, costs_total_weekly_fee</x:v>
+      </x:c>
+      <x:c r="E10" s="42" t="str">
+        <x:v>Contracted; cost is selected, payment fields are not</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="str">
+        <x:v>gold.fct_ipa[estimated_weekly_cost] only</x:v>
+      </x:c>
+      <x:c r="G10" s="42" t="str">
+        <x:v>Partially promoted</x:v>
+      </x:c>
+      <x:c r="H10" s="43" t="str">
+        <x:v>No new source file is needed. Add payment_method and approved finance fields only if payment reporting is in scope.</x:v>
+      </x:c>
+      <x:c r="I10" s="147" t="str">
+        <x:v>No — promote payment fact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="41" t="str">
+        <x:v>Child demographics</x:v>
+      </x:c>
+      <x:c r="B11" s="42" t="str">
+        <x:v>referral_person</x:v>
+      </x:c>
+      <x:c r="C11" s="42" t="str">
+        <x:v>bronze.referral_person → silver.referral_person</x:v>
+      </x:c>
+      <x:c r="D11" s="42" t="str">
+        <x:v>person_id, referral_id, gender, ethnicity, age_value</x:v>
+      </x:c>
+      <x:c r="E11" s="42" t="str">
+        <x:v>Contracted and used for child_id only</x:v>
+      </x:c>
+      <x:c r="F11" s="42" t="str">
+        <x:v>gold.fact_referral[child_id] only</x:v>
+      </x:c>
+      <x:c r="G11" s="42" t="str">
+        <x:v>Partially promoted</x:v>
+      </x:c>
+      <x:c r="H11" s="43" t="str">
+        <x:v>No new source file is needed. Publish a child/referral-person fact or dimension with agreed safeguarding controls.</x:v>
+      </x:c>
+      <x:c r="I11" s="147" t="str">
+        <x:v>No — promote child dimension</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="41" t="str">
+        <x:v>Child support needs</x:v>
+      </x:c>
+      <x:c r="B12" s="42" t="str">
+        <x:v>referral_person_support_needs</x:v>
+      </x:c>
+      <x:c r="C12" s="42" t="str">
+        <x:v>bronze.referral_person_support_needs → silver.referral_person_support_needs</x:v>
+      </x:c>
+      <x:c r="D12" s="42" t="str">
+        <x:v>person_id, support_need</x:v>
+      </x:c>
+      <x:c r="E12" s="42" t="str">
+        <x:v>Contracted; Silver formatter materialises it</x:v>
+      </x:c>
+      <x:c r="F12" s="42" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G12" s="42" t="str">
+        <x:v>Silver available — not promoted</x:v>
+      </x:c>
+      <x:c r="H12" s="43" t="str">
+        <x:v>Build a Gold bridge at person/referral-support-need grain before adding support-needs KPIs.</x:v>
+      </x:c>
+      <x:c r="I12" s="147" t="str">
+        <x:v>No — promote support-needs fact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="41" t="str">
+        <x:v>Referral categories</x:v>
+      </x:c>
+      <x:c r="B13" s="42" t="str">
+        <x:v>referral_category + framework_category</x:v>
+      </x:c>
+      <x:c r="C13" s="42" t="str">
+        <x:v>bronze.referral_category → silver.referral_category; silver.framework_category</x:v>
+      </x:c>
+      <x:c r="D13" s="42" t="str">
+        <x:v>referral_id, framework_category_id, category_name</x:v>
+      </x:c>
+      <x:c r="E13" s="42" t="str">
+        <x:v>Contracted; framework category is already modelled</x:v>
+      </x:c>
+      <x:c r="F13" s="42" t="str">
+        <x:v>gold.dim_framework_category only</x:v>
+      </x:c>
+      <x:c r="G13" s="42" t="str">
+        <x:v>Partially promoted</x:v>
+      </x:c>
+      <x:c r="H13" s="43" t="str">
+        <x:v>The referral-category assignment fact is not in Gold. Add a referral-category bridge/fact for category analysis and change history.</x:v>
+      </x:c>
+      <x:c r="I13" s="147" t="str">
+        <x:v>No — promote referral category</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="41" t="str">
+        <x:v>Provider messages</x:v>
+      </x:c>
+      <x:c r="B14" s="42" t="str">
+        <x:v>referral_provider_message</x:v>
+      </x:c>
+      <x:c r="C14" s="42" t="str">
+        <x:v>bronze.referral_provider_message → silver.referral_provider_message</x:v>
+      </x:c>
+      <x:c r="D14" s="42" t="str">
+        <x:v>message_id, referral_provider_id, created_timestamp, message_read_timestamp</x:v>
+      </x:c>
+      <x:c r="E14" s="42" t="str">
+        <x:v>Contracted; conditionally used by Silver lifecycle roll-up</x:v>
+      </x:c>
+      <x:c r="F14" s="42" t="str">
+        <x:v>gold.fact_referral_lifecycle_event (ProviderMessageSent event only)</x:v>
+      </x:c>
+      <x:c r="G14" s="42" t="str">
+        <x:v>Partially promoted</x:v>
+      </x:c>
+      <x:c r="H14" s="43" t="str">
+        <x:v>Message volume can be proxied by lifecycle events; response-time, unread and message-content analysis need a Gold message fact.</x:v>
+      </x:c>
+      <x:c r="I14" s="147" t="str">
+        <x:v>Yes — Gold lifecycle proxy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="41" t="str">
+        <x:v>Message read status</x:v>
+      </x:c>
+      <x:c r="B15" s="42" t="str">
+        <x:v>referral_provider_message_status</x:v>
+      </x:c>
+      <x:c r="C15" s="42" t="str">
+        <x:v>bronze.referral_provider_message_status → silver.referral_provider_message_status</x:v>
+      </x:c>
+      <x:c r="D15" s="42" t="str">
+        <x:v>message_id, message_read_by, message_read_timestamp</x:v>
+      </x:c>
+      <x:c r="E15" s="42" t="str">
+        <x:v>Source-capture mapping exists; validate contract/extract availability</x:v>
+      </x:c>
+      <x:c r="F15" s="42" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G15" s="42" t="str">
+        <x:v>Needs contract validation</x:v>
+      </x:c>
+      <x:c r="H15" s="43" t="str">
+        <x:v>Needed for unread/priority-message KPIs. Add to schema contract and Gold only after extract evidence is confirmed.</x:v>
+      </x:c>
+      <x:c r="I15" s="147" t="str">
+        <x:v>No — promote message-status fact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="41" t="str">
+        <x:v>Decline reasons</x:v>
+      </x:c>
+      <x:c r="B16" s="42" t="str">
+        <x:v>referral_provider_decline_reason</x:v>
+      </x:c>
+      <x:c r="C16" s="42" t="str">
+        <x:v>bronze.referral_provider_decline_reason → silver.referral_provider_decline_reason</x:v>
+      </x:c>
+      <x:c r="D16" s="42" t="str">
+        <x:v>decline_reason_id, referral_provider_id, decline_reason, created_date</x:v>
+      </x:c>
+      <x:c r="E16" s="42" t="str">
+        <x:v>Contracted; source FK retained</x:v>
+      </x:c>
+      <x:c r="F16" s="42" t="str">
+        <x:v>fact_offer[rejection_reason] is offer-level only</x:v>
+      </x:c>
+      <x:c r="G16" s="42" t="str">
+        <x:v>Silver available — not promoted</x:v>
+      </x:c>
+      <x:c r="H16" s="43" t="str">
+        <x:v>No new source file is needed. Build a Gold decline-reason fact joined through referral_provider for referral-level analysis.</x:v>
+      </x:c>
+      <x:c r="I16" s="147" t="str">
+        <x:v>No — promote decline-reason field</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="41" t="str">
+        <x:v>Provider documents</x:v>
+      </x:c>
+      <x:c r="B17" s="42" t="str">
+        <x:v>provider_submission_docs</x:v>
+      </x:c>
+      <x:c r="C17" s="42" t="str">
+        <x:v>bronze.provider_submission_docs → silver.provider_submission_docs</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="str">
+        <x:v>document_id, home_id, document_type, expiry_date, next_review_date</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="str">
+        <x:v>Contracted and used</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="str">
+        <x:v>gold.dim_provider_submission_document</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="str">
+        <x:v>Published in Gold</x:v>
+      </x:c>
+      <x:c r="H17" s="43" t="str">
+        <x:v>Expiry and expired-document measures are supported.</x:v>
+      </x:c>
+      <x:c r="I17" s="147" t="str">
+        <x:v>Yes — Gold field</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="41" t="str">
+        <x:v>Document compliance / blocking</x:v>
+      </x:c>
+      <x:c r="B18" s="42" t="str">
+        <x:v>Required-document policy and provider exclusion outcome</x:v>
+      </x:c>
+      <x:c r="C18" s="42" t="str">
+        <x:v>No confirmed source entity in the active contract</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="str">
+        <x:v>Expected document set, compliance result, blocked/excluded decision</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="str">
+        <x:v>Not supplied</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="str">
+        <x:v>New source required</x:v>
+      </x:c>
+      <x:c r="H18" s="43" t="str">
+        <x:v>Document dates alone cannot prove compliance or provider blocking; obtain the policy/decision data first.</x:v>
+      </x:c>
+      <x:c r="I18" s="147" t="str">
+        <x:v>No — new policy/outcome source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="41" t="str">
+        <x:v>Out-of-region</x:v>
+      </x:c>
+      <x:c r="B19" s="42" t="str">
+        <x:v>Referral region or out-of-region flag</x:v>
+      </x:c>
+      <x:c r="C19" s="42" t="str">
+        <x:v>No referral-level field in active schema_definition.csv</x:v>
+      </x:c>
+      <x:c r="D19" s="42" t="str">
+        <x:v>referral region, placement region or approved out-of-region flag</x:v>
+      </x:c>
+      <x:c r="E19" s="42" t="str">
+        <x:v>Not supplied</x:v>
+      </x:c>
+      <x:c r="F19" s="42" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G19" s="42" t="str">
+        <x:v>New source required</x:v>
+      </x:c>
+      <x:c r="H19" s="43" t="str">
+        <x:v>Provider county/country must not be used as a proxy for referral geography.</x:v>
+      </x:c>
+      <x:c r="I19" s="147" t="str">
+        <x:v>No — new referral geography source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="44" t="str">
+        <x:v>Framework change history</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="str">
+        <x:v>referral_category_aud (candidate)</x:v>
+      </x:c>
+      <x:c r="C20" s="45" t="str">
+        <x:v>bronze.referral_category_aud → silver.referral_category_aud</x:v>
+      </x:c>
+      <x:c r="D20" s="45" t="str">
+        <x:v>referral_id, framework_category_id, audit/change timestamp</x:v>
+      </x:c>
+      <x:c r="E20" s="45" t="str">
+        <x:v>Capture mapping exists; validate current extract and contract</x:v>
+      </x:c>
+      <x:c r="F20" s="45" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G20" s="45" t="str">
+        <x:v>Needs contract validation</x:v>
+      </x:c>
+      <x:c r="H20" s="46" t="str">
+        <x:v>Promote a category-history fact only after the audit table and change timestamp are confirmed.</x:v>
+      </x:c>
+      <x:c r="I20" s="147" t="str">
+        <x:v>No — validate then promote audit fact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21"/>
+    <x:row r="22"/>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="128" t="str">
+        <x:v>How to interpret Gold coverage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A24" s="130" t="str">
+        <x:v>Published in Gold</x:v>
+      </x:c>
+      <x:c r="B24" s="29" t="str">
+        <x:v>The source entity/fields are actively used in a current Gold fact, dimension or bridge.</x:v>
+      </x:c>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="31"/>
+    </x:row>
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="131" t="str">
+        <x:v>Partially promoted</x:v>
+      </x:c>
+      <x:c r="B25" s="32" t="str">
+        <x:v>Some relevant fields are in Gold, but the fields/grain required for the full requirement are not.</x:v>
+      </x:c>
+      <x:c r="C25" s="33"/>
+      <x:c r="D25" s="33"/>
+      <x:c r="E25" s="33"/>
+      <x:c r="F25" s="33"/>
+      <x:c r="G25" s="33"/>
+      <x:c r="H25" s="34"/>
+    </x:row>
+    <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A26" s="131" t="str">
+        <x:v>Silver available — not promoted</x:v>
+      </x:c>
+      <x:c r="B26" s="32" t="str">
+        <x:v>The source is contracted and expected in Silver; the Gold table/fact still needs to be created or extended.</x:v>
+      </x:c>
+      <x:c r="C26" s="33"/>
+      <x:c r="D26" s="33"/>
+      <x:c r="E26" s="33"/>
+      <x:c r="F26" s="33"/>
+      <x:c r="G26" s="33"/>
+      <x:c r="H26" s="34"/>
+    </x:row>
+    <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A27" s="131" t="str">
+        <x:v>Needs contract validation</x:v>
+      </x:c>
+      <x:c r="B27" s="32" t="str">
+        <x:v>A source capture mapping exists, but extract and contract evidence need validating before Gold is designed.</x:v>
+      </x:c>
+      <x:c r="C27" s="33"/>
+      <x:c r="D27" s="33"/>
+      <x:c r="E27" s="33"/>
+      <x:c r="F27" s="33"/>
+      <x:c r="G27" s="33"/>
+      <x:c r="H27" s="34"/>
+    </x:row>
+    <x:row r="28" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A28" s="132" t="str">
+        <x:v>New source required</x:v>
+      </x:c>
+      <x:c r="B28" s="35" t="str">
+        <x:v>No suitable field/entity exists in the active source contract; obtain or agree a new source first.</x:v>
+      </x:c>
+      <x:c r="C28" s="36"/>
+      <x:c r="D28" s="36"/>
+      <x:c r="E28" s="36"/>
+      <x:c r="F28" s="36"/>
+      <x:c r="G28" s="36"/>
+      <x:c r="H28" s="37"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A23:H23"/>
+    <x:mergeCell ref="A2:I2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G5:G20">
+    <x:cfRule type="containsText" dxfId="36" priority="1" operator="containsText" text="Published in Gold"/>
+    <x:cfRule type="containsText" dxfId="37" priority="2" operator="containsText" text="Partially promoted"/>
+    <x:cfRule type="containsText" dxfId="38" priority="3" operator="containsText" text="Silver available"/>
+    <x:cfRule type="containsText" dxfId="39" priority="4" operator="containsText" text="Needs contract validation"/>
+    <x:cfRule type="containsText" dxfId="40" priority="5" operator="containsText" text="New source required"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="A24:A28">
+    <x:cfRule type="containsText" dxfId="41" priority="6" operator="containsText" text="Published in Gold"/>
+    <x:cfRule type="containsText" dxfId="42" priority="7" operator="containsText" text="Partially promoted"/>
+    <x:cfRule type="containsText" dxfId="43" priority="8" operator="containsText" text="Silver available"/>
+    <x:cfRule type="containsText" dxfId="44" priority="9" operator="containsText" text="Needs contract validation"/>
+    <x:cfRule type="containsText" dxfId="45" priority="10" operator="containsText" text="New source required"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I5:I20">
+    <x:cfRule type="beginsWith" dxfId="46" priority="11" operator="beginsWith" text="Yes"/>
+    <x:cfRule type="beginsWith" dxfId="47" priority="12" operator="beginsWith" text="No"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7db55cd0d9a54a40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(gold): reconcile full legacy v15 measure library, port 76 DAX measures to Gold
</commit_message>
<xml_diff>
--- a/project X/configuration/Dashboard Legend.xlsx
+++ b/project X/configuration/Dashboard Legend.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R29673c5aae9e420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="Rfc5658c09e2e4a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="Rfa46288eb3004e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="R4a1ec47b108f4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="1" r:id="R4db792a30c7a43f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Definition" sheetId="2" r:id="Rf34252c1ff014cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definition" sheetId="4" r:id="R830e427a3dab4458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gold Source Coverage" sheetId="5" r:id="R2dce5f3603fd4bb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2011,7 +2011,7 @@
         <x:color rgb="FF1F4D2E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -2021,7 +2021,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -5654,7 +5654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6548377d9a764079"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15288ac76a114eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5701,7 +5701,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="100" t="str">
-        <x:v>Every Ready measure is defined in project X/client documentation/04_Data_and_Reporting/GOLD_SEMANTIC_MODEL_DAX_BUILD_GUIDE.md. These entries use only active Gold facts, dimensions and bridges; do not port legacy Bronze, Silver or retired fact references.</x:v>
+        <x:v>Current Gold-only DAX catalogue: 109 published measures (108 Ready, 1 lifecycle-event proxy), including Average Estimated Weekly Cost — Confirmed Referrals and Provider Messages Sent. End-to-end lineage: client documentation/04_Data_and_Reporting/KPI_Lineage.md.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -9439,8 +9439,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e89323d8ede4065"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2575e3d04b3646af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R127bfc275416499a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8073f206ba004aa2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10075,7 +10075,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7db55cd0d9a54a40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2e9218317854eac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>